<commit_message>
updates daily log for date --08/09/02026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\stash\daily_log\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CACED6F-4808-44BC-AFF7-F719C1900DC5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>26-09-03</t>
+  </si>
+  <si>
+    <t>learned packing and unpacking opearatosin python !</t>
   </si>
 </sst>
 </file>
@@ -1501,27 +1504,51 @@
       </c>
       <c r="N15" s="17"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>39717</v>
+      </c>
+      <c r="B16" s="14">
+        <v>400</v>
+      </c>
+      <c r="C16" s="14">
+        <v>10</v>
+      </c>
+      <c r="D16" s="14">
+        <v>200</v>
+      </c>
+      <c r="E16" s="14">
+        <v>400</v>
+      </c>
+      <c r="F16" s="14">
+        <v>300</v>
+      </c>
+      <c r="G16" s="14">
+        <v>6</v>
+      </c>
+      <c r="H16" s="14">
+        <v>10</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1320</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>120</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>

</xml_diff>

<commit_message>
updated daily logs for dates (08- annd 09)-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CACED6F-4808-44BC-AFF7-F719C1900DC5}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7B6FB33-5066-43FD-8B0D-1837EE0CA03A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>learned packing and unpacking opearatosin python !</t>
+  </si>
+  <si>
+    <t>started fucntions for python</t>
+  </si>
+  <si>
+    <t xml:space="preserve">continied functions for python </t>
   </si>
 </sst>
 </file>
@@ -1506,7 +1512,7 @@
     </row>
     <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
-        <v>39717</v>
+        <v>46273</v>
       </c>
       <c r="B16" s="14">
         <v>400</v>
@@ -1551,48 +1557,96 @@
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="A17" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B17" s="14">
+        <v>500</v>
+      </c>
+      <c r="C17" s="14">
+        <v>5</v>
+      </c>
+      <c r="D17" s="14">
+        <v>200</v>
+      </c>
+      <c r="E17" s="14">
+        <v>600</v>
+      </c>
+      <c r="F17" s="14">
+        <v>300</v>
+      </c>
+      <c r="G17" s="14">
+        <v>6</v>
+      </c>
+      <c r="H17" s="14">
+        <v>10</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>1615</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>-175</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B18" s="14">
+        <v>500</v>
+      </c>
+      <c r="C18" s="14">
+        <v>10</v>
+      </c>
+      <c r="D18" s="14">
+        <v>200</v>
+      </c>
+      <c r="E18" s="14">
+        <v>600</v>
+      </c>
+      <c r="F18" s="14">
+        <v>240</v>
+      </c>
+      <c r="G18" s="14">
+        <v>4</v>
+      </c>
+      <c r="H18" s="14">
+        <v>15</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1565</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>-125</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>

</xml_diff>

<commit_message>
updated daily logs for dates 11-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7B6FB33-5066-43FD-8B0D-1837EE0CA03A}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93DA531C-79A8-495B-A0B4-091FEC6AE807}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t xml:space="preserve">continied functions for python </t>
+  </si>
+  <si>
+    <t xml:space="preserve">continued functions for python </t>
   </si>
 </sst>
 </file>
@@ -1649,26 +1652,50 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B19" s="14">
+        <v>400</v>
+      </c>
+      <c r="C19" s="14">
+        <v>15</v>
+      </c>
+      <c r="D19" s="14">
+        <v>150</v>
+      </c>
+      <c r="E19" s="14">
+        <v>550</v>
+      </c>
+      <c r="F19" s="14">
+        <v>300</v>
+      </c>
+      <c r="G19" s="14">
+        <v>4</v>
+      </c>
+      <c r="H19" s="14">
+        <v>5</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1420</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>20</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="13"/>

</xml_diff>

<commit_message>
updated daily logs for dates 12-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93DA531C-79A8-495B-A0B4-091FEC6AE807}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1825C125-1AF9-4424-80DE-0CEE08E3D5CB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -280,6 +280,9 @@
   </si>
   <si>
     <t xml:space="preserve">continued functions for python </t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
   </si>
 </sst>
 </file>
@@ -1698,26 +1701,50 @@
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="13">
+        <v>41116</v>
+      </c>
+      <c r="B20" s="14">
+        <v>550</v>
+      </c>
+      <c r="C20" s="14">
+        <v>10</v>
+      </c>
+      <c r="D20" s="14">
+        <v>100</v>
+      </c>
+      <c r="E20" s="14">
+        <v>400</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14">
+        <v>10</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>370</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>

</xml_diff>

<commit_message>
updated daily logs for dates 13-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1825C125-1AF9-4424-80DE-0CEE08E3D5CB}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB74FF22-3A67-4470-8F2B-837E12125057}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1702,7 +1702,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
-        <v>41116</v>
+        <v>46215</v>
       </c>
       <c r="B20" s="14">
         <v>550</v>
@@ -1747,25 +1747,47 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B21" s="14">
+        <v>440</v>
+      </c>
+      <c r="C21" s="14">
+        <v>25</v>
+      </c>
+      <c r="D21" s="14">
+        <v>100</v>
+      </c>
+      <c r="E21" s="14">
+        <v>350</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14">
+        <v>0</v>
+      </c>
+      <c r="H21" s="14">
+        <v>15</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>930</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
+        <v>510</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>64</v>
+      </c>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated daily logs for dates 14-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB74FF22-3A67-4470-8F2B-837E12125057}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{024B7709-6742-45F6-84C0-F2D9A2E135CE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1791,25 +1791,47 @@
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B22" s="14">
+        <v>330</v>
+      </c>
+      <c r="C22" s="14">
+        <v>10</v>
+      </c>
+      <c r="D22" s="14">
+        <v>100</v>
+      </c>
+      <c r="E22" s="14">
+        <v>300</v>
+      </c>
+      <c r="F22" s="14">
+        <v>200</v>
+      </c>
+      <c r="G22" s="14">
+        <v>4</v>
+      </c>
+      <c r="H22" s="14">
+        <v>10</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated daily logs for dates 15-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{024B7709-6742-45F6-84C0-F2D9A2E135CE}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{961C722F-2ACE-4431-B544-0EB7AD64E43B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>2026-0915</t>
   </si>
 </sst>
 </file>
@@ -1835,25 +1838,47 @@
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="14">
+        <v>280</v>
+      </c>
+      <c r="C23" s="14">
+        <v>10</v>
+      </c>
+      <c r="D23" s="14">
+        <v>100</v>
+      </c>
+      <c r="E23" s="14">
+        <v>300</v>
+      </c>
+      <c r="F23" s="14">
+        <v>300</v>
+      </c>
+      <c r="G23" s="14">
+        <v>6</v>
+      </c>
+      <c r="H23" s="14">
+        <v>15</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1005</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
+        <v>435</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated daily logs for dates 18-09-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{961C722F-2ACE-4431-B544-0EB7AD64E43B}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17206E0A-26AB-49DD-BC65-75E6AF84E3CB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>2026-0915</t>
+  </si>
+  <si>
+    <t>Stressed</t>
   </si>
 </sst>
 </file>
@@ -959,7 +962,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1882,69 +1885,135 @@
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B24" s="14">
+        <v>200</v>
+      </c>
+      <c r="C24" s="14">
+        <v>20</v>
+      </c>
+      <c r="D24" s="14">
+        <v>10</v>
+      </c>
+      <c r="E24" s="14">
+        <v>300</v>
+      </c>
+      <c r="F24" s="14">
+        <v>420</v>
+      </c>
+      <c r="G24" s="14">
+        <v>7</v>
+      </c>
+      <c r="H24" s="14">
+        <v>45</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>995</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
+        <v>445</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>64</v>
+      </c>
       <c r="N24" s="17"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+      <c r="A25" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B25" s="14">
+        <v>400</v>
+      </c>
+      <c r="C25" s="14">
+        <v>15</v>
+      </c>
+      <c r="D25" s="14">
+        <v>200</v>
+      </c>
+      <c r="E25" s="14">
+        <v>150</v>
+      </c>
+      <c r="F25" s="14">
+        <v>250</v>
+      </c>
+      <c r="G25" s="14">
+        <v>5</v>
+      </c>
+      <c r="H25" s="14">
+        <v>11</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1026</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
+        <v>414</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N25" s="17"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+      <c r="A26" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B26" s="14">
+        <v>400</v>
+      </c>
+      <c r="C26" s="14">
+        <v>11</v>
+      </c>
+      <c r="D26" s="14">
+        <v>100</v>
+      </c>
+      <c r="E26" s="14">
+        <v>100</v>
+      </c>
+      <c r="F26" s="14">
+        <v>250</v>
+      </c>
+      <c r="G26" s="14">
+        <v>5</v>
+      </c>
+      <c r="H26" s="14">
+        <v>11</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>872</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
+        <v>568</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated lof for date:-2020/09/19
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17206E0A-26AB-49DD-BC65-75E6AF84E3CB}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C73D8A3-AD1B-44E2-A5FE-8D24DFEF768C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -289,6 +289,9 @@
   </si>
   <si>
     <t>Stressed</t>
+  </si>
+  <si>
+    <t>Excellent</t>
   </si>
 </sst>
 </file>
@@ -2017,25 +2020,47 @@
       <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+      <c r="A27" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B27" s="14">
+        <v>300</v>
+      </c>
+      <c r="C27" s="14">
+        <v>15</v>
+      </c>
+      <c r="D27" s="14">
+        <v>100</v>
+      </c>
+      <c r="E27" s="14">
+        <v>100</v>
+      </c>
+      <c r="F27" s="14">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14">
+        <v>0</v>
+      </c>
+      <c r="H27" s="14">
+        <v>10</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>525</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
+        <v>915</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated lof for date:-2020/09/20
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C73D8A3-AD1B-44E2-A5FE-8D24DFEF768C}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A337F637-B515-4020-803D-2AE8FF58D637}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2064,25 +2064,47 @@
       <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46285</v>
+      </c>
+      <c r="B28" s="14">
+        <v>250</v>
+      </c>
+      <c r="C28" s="14">
+        <v>10</v>
+      </c>
+      <c r="D28" s="14">
+        <v>100</v>
+      </c>
+      <c r="E28" s="14">
+        <v>200</v>
+      </c>
+      <c r="F28" s="14">
+        <v>0</v>
+      </c>
+      <c r="G28" s="14">
+        <v>0</v>
+      </c>
+      <c r="H28" s="14">
+        <v>10</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>570</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+        <v>870</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated lof for date:-2120/09/20
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A337F637-B515-4020-803D-2AE8FF58D637}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD885E2B-3A15-4C4B-BE26-2D54AB3DC26D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>Excellent</t>
+  </si>
+  <si>
+    <t>2026-0921</t>
   </si>
 </sst>
 </file>
@@ -2108,25 +2111,47 @@
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="14">
+        <v>200</v>
+      </c>
+      <c r="C29" s="14">
+        <v>10</v>
+      </c>
+      <c r="D29" s="14">
+        <v>200</v>
+      </c>
+      <c r="E29" s="14">
+        <v>100</v>
+      </c>
+      <c r="F29" s="14">
+        <v>150</v>
+      </c>
+      <c r="G29" s="14">
+        <v>3</v>
+      </c>
+      <c r="H29" s="14">
+        <v>10</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>670</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
+        <v>770</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>64</v>
+      </c>
       <c r="N29" s="17"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated lof for date:-22/09/20
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD885E2B-3A15-4C4B-BE26-2D54AB3DC26D}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1195F00-17DC-4C05-A72D-A93069AC6F87}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -292,9 +292,6 @@
   </si>
   <si>
     <t>Excellent</t>
-  </si>
-  <si>
-    <t>2026-0921</t>
   </si>
 </sst>
 </file>
@@ -2111,8 +2108,8 @@
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
-        <v>82</v>
+      <c r="A29" s="13">
+        <v>46286</v>
       </c>
       <c r="B29" s="14">
         <v>200</v>
@@ -2155,25 +2152,47 @@
       <c r="N29" s="17"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B30" s="14">
+        <v>150</v>
+      </c>
+      <c r="C30" s="14">
+        <v>12</v>
+      </c>
+      <c r="D30" s="14">
+        <v>200</v>
+      </c>
+      <c r="E30" s="14">
+        <v>100</v>
+      </c>
+      <c r="F30" s="14">
+        <v>300</v>
+      </c>
+      <c r="G30" s="14">
+        <v>6</v>
+      </c>
+      <c r="H30" s="14">
+        <v>10</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>772</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
+        <v>668</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N30" s="17"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated daily logs for date:
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="194" documentId="13_ncr:1_{1C9E7FEC-EE58-424A-AA43-67581D84C42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27B4C712-692E-46B7-8A21-6DEEC42DCE10}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{E5745785-2D17-4F37-A37C-5819BDC59475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AA67D2F-1D8B-4530-935B-D438AAA75EF9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,16 +17,11 @@
     <sheet name="Daily Log" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -109,6 +104,9 @@
     <t xml:space="preserve">   Notes               - short free-text note (exams, illness, travel, anything explaining an unusual day)</t>
   </si>
   <si>
+    <t>5. GOOD PRACTICE</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Fill this in at the same time every day (e.g. before bed) so entries stay accurate.</t>
   </si>
   <si>
@@ -121,13 +119,22 @@
     <t>Name:</t>
   </si>
   <si>
+    <t>DVV KARTHIK</t>
+  </si>
+  <si>
     <t>Registration No.:</t>
   </si>
   <si>
     <t>Course / Section:</t>
   </si>
   <si>
+    <t>MCA</t>
+  </si>
+  <si>
     <t>Month:</t>
+  </si>
+  <si>
+    <t>AUGUST</t>
   </si>
   <si>
     <t>All durations in MINUTES. Yellow cells = enter your data. Row 6 is a sample — overwrite it. Rows 2-3: fill your details.</t>
@@ -175,48 +182,16 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Satisfied</t>
+    <t>Neutral</t>
   </si>
   <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>5. GOOD PRACTICE</t>
+    <t>Satisfied</t>
   </si>
   <si>
-    <t>DVV KARTHIK</t>
-  </si>
-  <si>
-    <t>AUGUST</t>
-  </si>
-  <si>
-    <t>MCA</t>
-  </si>
-  <si>
-    <t>Neutral</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <u val="double"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Todyas pythons' learning</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>:- Extensively went deep into how and why the set data type is designed to posses the trait of "unorderly" arrangement of its constituent elements. Learned how it uses Hash Randomization, and a universal SipHash-2-4 algorithm to pass on a Unique Hash Address to its elements!!</t>
-    </r>
+    <t>Todyas pythons' learning:- Extensively went deep into how and why the set data type is designed to posses the trait of "unorderly" arrangement of its constituent elements. Learned how it uses Hash Randomization, and a universal SipHash-2-4 algorithm to pass on a Unique Hash Address to its elements!!</t>
   </si>
   <si>
     <t>Low</t>
@@ -237,16 +212,10 @@
     <t>learned for the pvm actually excecutes the function line by line for lists by creating a pylisobject in the heap!</t>
   </si>
   <si>
-    <t>26-07-29</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
     <t>learned  annd clarified a lot of doubts on the while loops in python and masterd  some more dictionary conprehensions!!</t>
-  </si>
-  <si>
-    <t>26-07-30</t>
   </si>
   <si>
     <t>Very Satisfied</t>
@@ -255,16 +224,13 @@
     <t>learnt the iterable filtering techniques like filter(), map(), and lambda functions!!</t>
   </si>
   <si>
-    <t>26-07-31</t>
-  </si>
-  <si>
     <t>learned whil eoopsloops and functions~!</t>
   </si>
   <si>
-    <t>learning how to use filter functions with def calls as their arguments!</t>
+    <t>26-09-02</t>
   </si>
   <si>
-    <t>26-09-02</t>
+    <t>learning how to use filter functions with def calls as their arguments!</t>
   </si>
   <si>
     <t>26-09-03</t>
@@ -298,8 +264,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="[$-14009]yyyy/mm/dd;@"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -383,14 +350,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
-      <u val="double"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -402,6 +361,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -425,7 +391,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -448,11 +414,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -493,16 +483,25 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -786,12 +785,12 @@
     <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="22.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -938,17 +937,17 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
@@ -965,7 +964,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -986,117 +985,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
+      <c r="A1" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+        <v>31</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="26"/>
       <c r="E2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="23">
+        <v>33</v>
+      </c>
+      <c r="F2" s="25">
         <v>12620739</v>
       </c>
-      <c r="G2" s="23"/>
+      <c r="G2" s="26"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
+        <v>34</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="27"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" s="23"/>
+        <v>36</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-    </row>
-    <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>35</v>
+      <c r="A4" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+    </row>
+    <row r="5" spans="1:14" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>39</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -1115,67 +1114,65 @@
       <c r="M6" s="11"/>
       <c r="N6" s="12"/>
     </row>
-    <row r="7" spans="1:14" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="18">
-        <v>46228</v>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
+        <v>46253</v>
       </c>
       <c r="B7" s="14">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C7" s="14">
         <v>15</v>
       </c>
       <c r="D7" s="14">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="E7" s="14">
+        <v>200</v>
+      </c>
+      <c r="F7" s="14">
         <v>300</v>
       </c>
-      <c r="F7" s="14">
-        <v>100</v>
-      </c>
       <c r="G7" s="14">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H7" s="14">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="I7" s="15">
-        <f t="shared" ref="I7:I69" si="0">IF(SUM(B7:F7,H7)=0,"",SUM(B7:F7,H7))</f>
-        <v>980</v>
+        <f t="shared" ref="I7:I70" si="0">IF(SUM(B7:F7,H7)=0,"",SUM(B7:F7,H7))</f>
+        <v>1030</v>
       </c>
       <c r="J7" s="15">
-        <f t="shared" ref="J7:J69" si="1">IF(I7="","",1440-I7)</f>
-        <v>460</v>
+        <f t="shared" ref="J7:J70" si="1">IF(I7="","",1440-I7)</f>
+        <v>410</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N7" s="19" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+      <c r="N7" s="17"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
-        <v>46229</v>
+        <v>46254</v>
       </c>
       <c r="B8" s="14">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="C8" s="14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D8" s="14">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E8" s="14">
-        <v>420</v>
+        <v>150</v>
       </c>
       <c r="F8" s="14">
         <v>150</v>
@@ -1184,263 +1181,253 @@
         <v>3</v>
       </c>
       <c r="H8" s="14">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v>1015</v>
+        <v>875</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v>425</v>
+        <v>565</v>
       </c>
       <c r="K8" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="16" t="s">
-        <v>49</v>
-      </c>
       <c r="M8" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N8" s="20" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="N8" s="17"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
-        <v>46230</v>
+        <v>46255</v>
       </c>
       <c r="B9" s="14">
-        <v>400</v>
+        <v>550</v>
       </c>
       <c r="C9" s="14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D9" s="14">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="E9" s="14">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="F9" s="14">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G9" s="14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H9" s="14">
         <v>15</v>
       </c>
       <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v>1135</v>
+        <v>1275</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v>305</v>
+        <v>165</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+      <c r="N9" s="17"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
-        <v>46231</v>
+        <v>46256</v>
       </c>
       <c r="B10" s="14">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C10" s="14">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D10" s="14">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="E10" s="14">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F10" s="14">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="G10" s="14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" s="14">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v>1275</v>
+        <v>970</v>
       </c>
       <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v>165</v>
+        <v>470</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
-        <v>63</v>
+        <v>57</v>
+      </c>
+      <c r="N10" s="17"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>46257</v>
       </c>
       <c r="B11" s="14">
-        <v>450</v>
+        <v>330</v>
       </c>
       <c r="C11" s="14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D11" s="14">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E11" s="14">
-        <v>420</v>
+        <v>250</v>
       </c>
       <c r="F11" s="14">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="G11" s="14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H11" s="14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v>1030</v>
+        <v>950</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v>410</v>
+        <v>490</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="N11" s="17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
-        <v>66</v>
+        <v>54</v>
+      </c>
+      <c r="N11" s="17"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>46258</v>
       </c>
       <c r="B12" s="14">
-        <v>500</v>
+        <v>280</v>
       </c>
       <c r="C12" s="14">
+        <v>10</v>
+      </c>
+      <c r="D12" s="14">
+        <v>100</v>
+      </c>
+      <c r="E12" s="14">
+        <v>200</v>
+      </c>
+      <c r="F12" s="14">
+        <v>200</v>
+      </c>
+      <c r="G12" s="14">
+        <v>4</v>
+      </c>
+      <c r="H12" s="14">
         <v>15</v>
-      </c>
-      <c r="D12" s="14">
-        <v>200</v>
-      </c>
-      <c r="E12" s="14">
-        <v>500</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14">
-        <v>5</v>
       </c>
       <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v>1220</v>
+        <v>805</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>635</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="N12" s="17" t="s">
-        <v>68</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
-        <v>69</v>
+      <c r="A13" s="13">
+        <v>46263</v>
       </c>
       <c r="B13" s="14">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="C13" s="14">
+        <v>20</v>
+      </c>
+      <c r="D13" s="14">
         <v>10</v>
       </c>
-      <c r="D13" s="14">
-        <v>200</v>
-      </c>
       <c r="E13" s="14">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F13" s="14">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G13" s="14">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H13" s="14">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v>1225</v>
+        <v>840</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v>215</v>
+        <v>600</v>
       </c>
       <c r="K13" s="16" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
-        <v>72</v>
+        <v>54</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N13" s="17"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <v>46264</v>
       </c>
       <c r="B14" s="14">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="C14" s="14">
         <v>15</v>
@@ -1458,88 +1445,86 @@
         <v>5</v>
       </c>
       <c r="H14" s="14">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v>1085</v>
+        <v>1130</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v>355</v>
+        <v>310</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N14" s="17" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
-        <v>73</v>
+        <v>54</v>
+      </c>
+      <c r="N14" s="17"/>
+    </row>
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <v>46265</v>
       </c>
       <c r="B15" s="14">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="C15" s="14">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D15" s="14">
+        <v>100</v>
+      </c>
+      <c r="E15" s="14">
         <v>150</v>
       </c>
-      <c r="E15" s="14">
-        <v>300</v>
-      </c>
       <c r="F15" s="14">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="G15" s="14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15" s="14">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v>1135</v>
+        <v>856</v>
       </c>
       <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v>305</v>
+        <v>584</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>57</v>
       </c>
       <c r="N15" s="17"/>
     </row>
-    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
-        <v>46273</v>
+        <v>46266</v>
       </c>
       <c r="B16" s="14">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="C16" s="14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D16" s="14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E16" s="14">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F16" s="14">
         <v>300</v>
@@ -1548,228 +1533,226 @@
         <v>6</v>
       </c>
       <c r="H16" s="14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v>1320</v>
+        <v>1026</v>
       </c>
       <c r="J16" s="15">
         <f t="shared" si="1"/>
+        <v>414</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N16" s="17"/>
+    </row>
+    <row r="17" spans="1:14" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="21">
+        <v>46259</v>
+      </c>
+      <c r="B17" s="14">
+        <v>420</v>
+      </c>
+      <c r="C17" s="14">
+        <v>15</v>
+      </c>
+      <c r="D17" s="14">
         <v>120</v>
       </c>
-      <c r="K16" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="L16" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="M16" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N16" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13">
-        <v>46274</v>
-      </c>
-      <c r="B17" s="14">
-        <v>500</v>
-      </c>
-      <c r="C17" s="14">
-        <v>5</v>
-      </c>
-      <c r="D17" s="14">
-        <v>200</v>
-      </c>
       <c r="E17" s="14">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F17" s="14">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="G17" s="14">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H17" s="14">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v>1615</v>
+        <v>980</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v>-175</v>
+        <v>460</v>
       </c>
       <c r="K17" s="16" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N17" s="17" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13">
-        <v>46275</v>
+        <v>54</v>
+      </c>
+      <c r="N17" s="18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="22">
+        <v>46260</v>
       </c>
       <c r="B18" s="14">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="C18" s="14">
         <v>10</v>
       </c>
       <c r="D18" s="14">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="E18" s="14">
-        <v>600</v>
+        <v>420</v>
       </c>
       <c r="F18" s="14">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="G18" s="14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18" s="14">
         <v>15</v>
       </c>
       <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v>1565</v>
+        <v>1015</v>
       </c>
       <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v>-125</v>
+        <v>425</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L18" s="16" t="s">
         <v>55</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N18" s="17" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13">
-        <v>46276</v>
+        <v>54</v>
+      </c>
+      <c r="N18" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="22">
+        <v>46261</v>
       </c>
       <c r="B19" s="14">
         <v>400</v>
       </c>
       <c r="C19" s="14">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D19" s="14">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="E19" s="14">
-        <v>550</v>
+        <v>250</v>
       </c>
       <c r="F19" s="14">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G19" s="14">
         <v>4</v>
       </c>
       <c r="H19" s="14">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v>1420</v>
+        <v>1135</v>
       </c>
       <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>305</v>
       </c>
       <c r="K19" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13">
-        <v>46215</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="22">
+        <v>46262</v>
       </c>
       <c r="B20" s="14">
-        <v>550</v>
+        <v>450</v>
       </c>
       <c r="C20" s="14">
         <v>10</v>
       </c>
       <c r="D20" s="14">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="E20" s="14">
         <v>400</v>
       </c>
       <c r="F20" s="14">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="G20" s="14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H20" s="14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v>1070</v>
+        <v>1275</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v>370</v>
+        <v>165</v>
       </c>
       <c r="K20" s="16" t="s">
         <v>59</v>
       </c>
       <c r="L20" s="16" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13">
-        <v>46278</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="22">
+        <v>47356</v>
       </c>
       <c r="B21" s="14">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="C21" s="14">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D21" s="14">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E21" s="14">
-        <v>350</v>
+        <v>420</v>
       </c>
       <c r="F21" s="14">
         <v>0</v>
@@ -1778,993 +1761,1451 @@
         <v>0</v>
       </c>
       <c r="H21" s="14">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v>930</v>
+        <v>1030</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v>510</v>
+        <v>410</v>
       </c>
       <c r="K21" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L21" s="16" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="M21" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N21" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13">
-        <v>46279</v>
+    </row>
+    <row r="22" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="22">
+        <v>47721</v>
       </c>
       <c r="B22" s="14">
-        <v>330</v>
+        <v>500</v>
       </c>
       <c r="C22" s="14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D22" s="14">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E22" s="14">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="F22" s="14">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G22" s="14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H22" s="14">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v>950</v>
+        <v>1220</v>
       </c>
       <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v>490</v>
+        <v>220</v>
       </c>
       <c r="K22" s="16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L22" s="16" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N22" s="17"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
-        <v>79</v>
+        <v>63</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="22">
+        <v>48086</v>
       </c>
       <c r="B23" s="14">
-        <v>280</v>
+        <v>400</v>
       </c>
       <c r="C23" s="14">
         <v>10</v>
       </c>
       <c r="D23" s="14">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E23" s="14">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="F23" s="14">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G23" s="14">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H23" s="14">
         <v>15</v>
       </c>
       <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v>1005</v>
+        <v>1225</v>
       </c>
       <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v>435</v>
+        <v>215</v>
       </c>
       <c r="K23" s="16" t="s">
         <v>59</v>
       </c>
       <c r="L23" s="16" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N23" s="17"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13">
-        <v>46281</v>
+        <v>54</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="22" t="s">
+        <v>68</v>
       </c>
       <c r="B24" s="14">
+        <v>350</v>
+      </c>
+      <c r="C24" s="14">
+        <v>15</v>
+      </c>
+      <c r="D24" s="14">
         <v>200</v>
       </c>
-      <c r="C24" s="14">
+      <c r="E24" s="14">
+        <v>250</v>
+      </c>
+      <c r="F24" s="14">
+        <v>250</v>
+      </c>
+      <c r="G24" s="14">
+        <v>5</v>
+      </c>
+      <c r="H24" s="14">
         <v>20</v>
-      </c>
-      <c r="D24" s="14">
-        <v>10</v>
-      </c>
-      <c r="E24" s="14">
-        <v>300</v>
-      </c>
-      <c r="F24" s="14">
-        <v>420</v>
-      </c>
-      <c r="G24" s="14">
-        <v>7</v>
-      </c>
-      <c r="H24" s="14">
-        <v>45</v>
       </c>
       <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v>995</v>
+        <v>1085</v>
       </c>
       <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v>445</v>
+        <v>355</v>
       </c>
       <c r="K24" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L24" s="16" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="M24" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="N24" s="17"/>
+        <v>57</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13">
-        <v>46282</v>
+      <c r="A25" s="22" t="s">
+        <v>70</v>
       </c>
       <c r="B25" s="14">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="C25" s="14">
         <v>15</v>
       </c>
       <c r="D25" s="14">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E25" s="14">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="F25" s="14">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="G25" s="14">
         <v>5</v>
       </c>
       <c r="H25" s="14">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v>1026</v>
+        <v>1135</v>
       </c>
       <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v>414</v>
-      </c>
-      <c r="K25" s="16" t="s">
-        <v>59</v>
+        <v>305</v>
+      </c>
+      <c r="K25" s="14">
+        <v>10</v>
       </c>
       <c r="L25" s="16" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="M25" s="16" t="s">
         <v>57</v>
       </c>
       <c r="N25" s="17"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13">
-        <v>46283</v>
+    <row r="26" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="22">
+        <v>46273</v>
       </c>
       <c r="B26" s="14">
         <v>400</v>
       </c>
       <c r="C26" s="14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D26" s="14">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E26" s="14">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="F26" s="14">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="G26" s="14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H26" s="14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v>872</v>
+        <v>1320</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v>568</v>
-      </c>
-      <c r="K26" s="16" t="s">
-        <v>80</v>
+        <v>120</v>
+      </c>
+      <c r="K26" s="14">
+        <v>15</v>
       </c>
       <c r="L26" s="16" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="M26" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="N26" s="17"/>
+      <c r="N26" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13">
-        <v>46284</v>
+      <c r="A27" s="22">
+        <v>46274</v>
       </c>
       <c r="B27" s="14">
+        <v>500</v>
+      </c>
+      <c r="C27" s="14">
+        <v>5</v>
+      </c>
+      <c r="D27" s="14">
+        <v>200</v>
+      </c>
+      <c r="E27" s="14">
+        <v>600</v>
+      </c>
+      <c r="F27" s="14">
         <v>300</v>
       </c>
-      <c r="C27" s="14">
-        <v>15</v>
-      </c>
-      <c r="D27" s="14">
-        <v>100</v>
-      </c>
-      <c r="E27" s="14">
-        <v>100</v>
-      </c>
-      <c r="F27" s="14">
-        <v>0</v>
-      </c>
       <c r="G27" s="14">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H27" s="14">
         <v>10</v>
       </c>
       <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v>525</v>
+        <v>1615</v>
       </c>
       <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v>915</v>
-      </c>
-      <c r="K27" s="16" t="s">
-        <v>81</v>
+        <v>-175</v>
+      </c>
+      <c r="K27" s="14">
+        <v>5</v>
       </c>
       <c r="L27" s="16" t="s">
         <v>61</v>
       </c>
       <c r="M27" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N27" s="17"/>
+        <v>54</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13">
-        <v>46285</v>
+      <c r="A28" s="22">
+        <v>46275</v>
       </c>
       <c r="B28" s="14">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="C28" s="14">
         <v>10</v>
       </c>
       <c r="D28" s="14">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E28" s="14">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="F28" s="14">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="G28" s="14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H28" s="14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v>570</v>
+        <v>1565</v>
       </c>
       <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v>870</v>
-      </c>
-      <c r="K28" s="16" t="s">
-        <v>57</v>
+        <v>-125</v>
+      </c>
+      <c r="K28" s="14">
+        <v>10</v>
       </c>
       <c r="L28" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M28" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N28" s="17"/>
+        <v>54</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13">
-        <v>46286</v>
+      <c r="A29" s="22">
+        <v>46276</v>
       </c>
       <c r="B29" s="14">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="C29" s="14">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="D29" s="14">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E29" s="14">
-        <v>100</v>
+        <v>550</v>
       </c>
       <c r="F29" s="14">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="G29" s="14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H29" s="14">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v>670</v>
+        <v>1555</v>
       </c>
       <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v>770</v>
-      </c>
-      <c r="K29" s="16" t="s">
-        <v>55</v>
+        <v>-115</v>
+      </c>
+      <c r="K29" s="14">
+        <v>15</v>
       </c>
       <c r="L29" s="16" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="N29" s="17"/>
+        <v>57</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13">
-        <v>46287</v>
+      <c r="A30" s="22">
+        <v>46246</v>
       </c>
       <c r="B30" s="14">
-        <v>150</v>
+        <v>550</v>
       </c>
       <c r="C30" s="14">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D30" s="14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E30" s="14">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="F30" s="14">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G30" s="14">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H30" s="14">
         <v>10</v>
       </c>
       <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v>772</v>
+        <v>1070</v>
       </c>
       <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v>668</v>
-      </c>
-      <c r="K30" s="16" t="s">
-        <v>55</v>
+        <v>370</v>
+      </c>
+      <c r="K30" s="14">
+        <v>10</v>
       </c>
       <c r="L30" s="16" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="M30" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N30" s="17"/>
+        <v>54</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13">
-        <v>46288</v>
+      <c r="A31" s="22">
+        <v>46278</v>
       </c>
       <c r="B31" s="14">
-        <v>200</v>
+        <v>440</v>
       </c>
       <c r="C31" s="14">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D31" s="14">
         <v>100</v>
       </c>
       <c r="E31" s="14">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="F31" s="14">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G31" s="14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H31" s="14">
         <v>15</v>
       </c>
       <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v>729</v>
+        <v>930</v>
       </c>
       <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v>711</v>
-      </c>
-      <c r="K31" s="16" t="s">
-        <v>57</v>
+        <v>510</v>
+      </c>
+      <c r="K31" s="14">
+        <v>15</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="M31" s="16" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N31" s="17"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13">
-        <v>46289</v>
+      <c r="A32" s="22">
+        <v>46279</v>
       </c>
       <c r="B32" s="14">
+        <v>330</v>
+      </c>
+      <c r="C32" s="14">
+        <v>10</v>
+      </c>
+      <c r="D32" s="14">
+        <v>100</v>
+      </c>
+      <c r="E32" s="14">
+        <v>300</v>
+      </c>
+      <c r="F32" s="14">
         <v>200</v>
       </c>
-      <c r="C32" s="14">
-        <v>18</v>
-      </c>
-      <c r="D32" s="14">
-        <v>200</v>
-      </c>
-      <c r="E32" s="14">
-        <v>100</v>
-      </c>
-      <c r="F32" s="14">
-        <v>250</v>
-      </c>
       <c r="G32" s="14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H32" s="14">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v>793</v>
+        <v>950</v>
       </c>
       <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v>647</v>
-      </c>
-      <c r="K32" s="16" t="s">
-        <v>59</v>
+        <v>490</v>
+      </c>
+      <c r="K32" s="14">
+        <v>45</v>
       </c>
       <c r="L32" s="16" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="M32" s="16" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="N32" s="17"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13">
-        <v>46290</v>
+      <c r="A33" s="22" t="s">
+        <v>76</v>
       </c>
       <c r="B33" s="14">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="C33" s="14">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D33" s="14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E33" s="14">
         <v>300</v>
       </c>
       <c r="F33" s="14">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G33" s="14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H33" s="14">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v>915</v>
+        <v>1005</v>
       </c>
       <c r="J33" s="15">
         <f t="shared" si="1"/>
+        <v>435</v>
+      </c>
+      <c r="K33" s="14">
+        <v>11</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N33" s="17"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" s="22">
+        <v>46281</v>
+      </c>
+      <c r="B34" s="14">
+        <v>200</v>
+      </c>
+      <c r="C34" s="14">
+        <v>20</v>
+      </c>
+      <c r="D34" s="14">
+        <v>10</v>
+      </c>
+      <c r="E34" s="14">
+        <v>300</v>
+      </c>
+      <c r="F34" s="14">
+        <v>420</v>
+      </c>
+      <c r="G34" s="14">
+        <v>7</v>
+      </c>
+      <c r="H34" s="14">
+        <v>45</v>
+      </c>
+      <c r="I34" s="15">
+        <f t="shared" si="0"/>
+        <v>995</v>
+      </c>
+      <c r="J34" s="15">
+        <f t="shared" si="1"/>
+        <v>445</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N34" s="17"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" s="22">
+        <v>46282</v>
+      </c>
+      <c r="B35" s="14">
+        <v>400</v>
+      </c>
+      <c r="C35" s="14">
+        <v>15</v>
+      </c>
+      <c r="D35" s="14">
+        <v>200</v>
+      </c>
+      <c r="E35" s="14">
+        <v>150</v>
+      </c>
+      <c r="F35" s="14">
+        <v>250</v>
+      </c>
+      <c r="G35" s="14">
+        <v>5</v>
+      </c>
+      <c r="H35" s="14">
+        <v>11</v>
+      </c>
+      <c r="I35" s="15">
+        <f t="shared" si="0"/>
+        <v>1026</v>
+      </c>
+      <c r="J35" s="15">
+        <f t="shared" si="1"/>
+        <v>414</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N35" s="17"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="22">
+        <v>46283</v>
+      </c>
+      <c r="B36" s="14">
+        <v>400</v>
+      </c>
+      <c r="C36" s="14">
+        <v>11</v>
+      </c>
+      <c r="D36" s="14">
+        <v>100</v>
+      </c>
+      <c r="E36" s="14">
+        <v>100</v>
+      </c>
+      <c r="F36" s="14">
+        <v>250</v>
+      </c>
+      <c r="G36" s="14">
+        <v>5</v>
+      </c>
+      <c r="H36" s="14">
+        <v>11</v>
+      </c>
+      <c r="I36" s="15">
+        <f t="shared" si="0"/>
+        <v>872</v>
+      </c>
+      <c r="J36" s="15">
+        <f t="shared" si="1"/>
+        <v>568</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N36" s="17"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" s="22">
+        <v>46284</v>
+      </c>
+      <c r="B37" s="14">
+        <v>300</v>
+      </c>
+      <c r="C37" s="14">
+        <v>15</v>
+      </c>
+      <c r="D37" s="14">
+        <v>100</v>
+      </c>
+      <c r="E37" s="14">
+        <v>100</v>
+      </c>
+      <c r="F37" s="14">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14">
+        <v>10</v>
+      </c>
+      <c r="I37" s="15">
+        <f t="shared" si="0"/>
         <v>525</v>
       </c>
-      <c r="K33" s="16" t="s">
+      <c r="J37" s="15">
+        <f t="shared" si="1"/>
+        <v>915</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N37" s="17"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A38" s="22">
+        <v>46285</v>
+      </c>
+      <c r="B38" s="14">
+        <v>250</v>
+      </c>
+      <c r="C38" s="14">
+        <v>10</v>
+      </c>
+      <c r="D38" s="14">
+        <v>100</v>
+      </c>
+      <c r="E38" s="14">
+        <v>200</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>10</v>
+      </c>
+      <c r="I38" s="15">
+        <f t="shared" si="0"/>
+        <v>570</v>
+      </c>
+      <c r="J38" s="15">
+        <f t="shared" si="1"/>
+        <v>870</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N38" s="17"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A39" s="22">
+        <v>46286</v>
+      </c>
+      <c r="B39" s="14">
+        <v>200</v>
+      </c>
+      <c r="C39" s="14">
+        <v>10</v>
+      </c>
+      <c r="D39" s="14">
+        <v>200</v>
+      </c>
+      <c r="E39" s="14">
+        <v>100</v>
+      </c>
+      <c r="F39" s="14">
+        <v>150</v>
+      </c>
+      <c r="G39" s="14">
+        <v>3</v>
+      </c>
+      <c r="H39" s="14">
+        <v>10</v>
+      </c>
+      <c r="I39" s="15">
+        <f t="shared" si="0"/>
+        <v>670</v>
+      </c>
+      <c r="J39" s="15">
+        <f t="shared" si="1"/>
+        <v>770</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N39" s="17"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" s="22">
+        <v>46287</v>
+      </c>
+      <c r="B40" s="14">
+        <v>150</v>
+      </c>
+      <c r="C40" s="14">
+        <v>12</v>
+      </c>
+      <c r="D40" s="14">
+        <v>200</v>
+      </c>
+      <c r="E40" s="14">
+        <v>100</v>
+      </c>
+      <c r="F40" s="14">
+        <v>300</v>
+      </c>
+      <c r="G40" s="14">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14">
+        <v>10</v>
+      </c>
+      <c r="I40" s="15">
+        <f t="shared" si="0"/>
+        <v>772</v>
+      </c>
+      <c r="J40" s="15">
+        <f t="shared" si="1"/>
+        <v>668</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N40" s="17"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A41" s="22">
+        <v>46288</v>
+      </c>
+      <c r="B41" s="14">
+        <v>200</v>
+      </c>
+      <c r="C41" s="14">
+        <v>14</v>
+      </c>
+      <c r="D41" s="14">
+        <v>100</v>
+      </c>
+      <c r="E41" s="14">
+        <v>200</v>
+      </c>
+      <c r="F41" s="14">
+        <v>200</v>
+      </c>
+      <c r="G41" s="14">
+        <v>4</v>
+      </c>
+      <c r="H41" s="14">
+        <v>15</v>
+      </c>
+      <c r="I41" s="15">
+        <f t="shared" si="0"/>
+        <v>729</v>
+      </c>
+      <c r="J41" s="15">
+        <f t="shared" si="1"/>
+        <v>711</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N41" s="17"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A42" s="22">
+        <v>46289</v>
+      </c>
+      <c r="B42" s="14">
+        <v>200</v>
+      </c>
+      <c r="C42" s="14">
+        <v>18</v>
+      </c>
+      <c r="D42" s="14">
+        <v>200</v>
+      </c>
+      <c r="E42" s="14">
+        <v>100</v>
+      </c>
+      <c r="F42" s="14">
+        <v>250</v>
+      </c>
+      <c r="G42" s="14">
+        <v>5</v>
+      </c>
+      <c r="H42" s="14">
+        <v>25</v>
+      </c>
+      <c r="I42" s="15">
+        <f t="shared" si="0"/>
+        <v>793</v>
+      </c>
+      <c r="J42" s="15">
+        <f t="shared" si="1"/>
+        <v>647</v>
+      </c>
+      <c r="K42" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="L33" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="M33" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N33" s="17"/>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="L42" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N42" s="17"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" s="22">
+        <v>46290</v>
+      </c>
+      <c r="B43" s="14">
+        <v>200</v>
+      </c>
+      <c r="C43" s="14">
+        <v>7</v>
+      </c>
+      <c r="D43" s="14">
+        <v>200</v>
+      </c>
+      <c r="E43" s="14">
+        <v>300</v>
+      </c>
+      <c r="F43" s="14">
+        <v>200</v>
+      </c>
+      <c r="G43" s="14">
+        <v>4</v>
+      </c>
+      <c r="H43" s="14">
+        <v>8</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>915</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+        <v>525</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N43" s="17"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A44" s="22">
+        <v>46291</v>
+      </c>
+      <c r="B44" s="14">
+        <v>350</v>
+      </c>
+      <c r="C44" s="14">
+        <v>15</v>
+      </c>
+      <c r="D44" s="14">
+        <v>250</v>
+      </c>
+      <c r="E44" s="14">
+        <v>400</v>
+      </c>
+      <c r="F44" s="14">
+        <v>300</v>
+      </c>
+      <c r="G44" s="14">
+        <v>6</v>
+      </c>
+      <c r="H44" s="14">
+        <v>11</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1326</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+        <v>114</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N44" s="17"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" s="22">
+        <v>46292</v>
+      </c>
+      <c r="B45" s="14">
+        <v>280</v>
+      </c>
+      <c r="C45" s="14">
+        <v>25</v>
+      </c>
+      <c r="D45" s="14">
+        <v>300</v>
+      </c>
+      <c r="E45" s="14">
+        <v>400</v>
+      </c>
+      <c r="F45" s="14">
+        <v>250</v>
+      </c>
+      <c r="G45" s="14">
+        <v>5</v>
+      </c>
+      <c r="H45" s="14">
+        <v>10</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1265</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+        <v>175</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N45" s="17"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" s="22">
+        <v>46293</v>
+      </c>
+      <c r="B46" s="14">
+        <v>320</v>
+      </c>
+      <c r="C46" s="14">
+        <v>30</v>
+      </c>
+      <c r="D46" s="14">
+        <v>250</v>
+      </c>
+      <c r="E46" s="14">
+        <v>400</v>
+      </c>
+      <c r="F46" s="14">
+        <v>150</v>
+      </c>
+      <c r="G46" s="14">
+        <v>3</v>
+      </c>
+      <c r="H46" s="14">
+        <v>9</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>1159</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+        <v>281</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N46" s="17"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B47" s="14">
+        <v>225</v>
+      </c>
+      <c r="C47" s="14">
+        <v>11</v>
+      </c>
+      <c r="D47" s="14">
+        <v>310</v>
+      </c>
+      <c r="E47" s="14">
+        <v>400</v>
+      </c>
+      <c r="F47" s="14">
+        <v>300</v>
+      </c>
+      <c r="G47" s="14">
+        <v>6</v>
+      </c>
+      <c r="H47" s="14">
+        <v>15</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1261</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+        <v>179</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N47" s="17"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46295</v>
+      </c>
+      <c r="B48" s="14">
+        <v>310</v>
+      </c>
+      <c r="C48" s="14">
+        <v>9</v>
+      </c>
+      <c r="D48" s="14">
+        <v>285</v>
+      </c>
+      <c r="E48" s="14">
+        <v>400</v>
+      </c>
+      <c r="F48" s="14">
+        <v>350</v>
+      </c>
+      <c r="G48" s="14">
+        <v>7</v>
+      </c>
+      <c r="H48" s="14">
+        <v>12</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1366</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+        <v>74</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N48" s="17"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A49" s="13">
+        <v>46296</v>
+      </c>
+      <c r="B49" s="14">
+        <v>300</v>
+      </c>
+      <c r="C49" s="14">
+        <v>14</v>
+      </c>
+      <c r="D49" s="14">
+        <v>264</v>
+      </c>
+      <c r="E49" s="14">
+        <v>400</v>
+      </c>
+      <c r="F49" s="14">
+        <v>300</v>
+      </c>
+      <c r="G49" s="14">
+        <v>6</v>
+      </c>
+      <c r="H49" s="14">
+        <v>14</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1292</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+        <v>148</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N49" s="17"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B50" s="14">
+        <v>205</v>
+      </c>
+      <c r="C50" s="14">
+        <v>5</v>
+      </c>
+      <c r="D50" s="14">
+        <v>260</v>
+      </c>
+      <c r="E50" s="14">
+        <v>400</v>
+      </c>
+      <c r="F50" s="14">
+        <v>200</v>
+      </c>
+      <c r="G50" s="14">
+        <v>4</v>
+      </c>
+      <c r="H50" s="14">
+        <v>10</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+        <v>360</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N50" s="17"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A51" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B51" s="14">
+        <v>260</v>
+      </c>
+      <c r="C51" s="14">
+        <v>5</v>
+      </c>
+      <c r="D51" s="14">
+        <v>250</v>
+      </c>
+      <c r="E51" s="14">
+        <v>400</v>
+      </c>
+      <c r="F51" s="14">
+        <v>250</v>
+      </c>
+      <c r="G51" s="14">
+        <v>5</v>
+      </c>
+      <c r="H51" s="14">
+        <v>11</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>1176</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+        <v>264</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N51" s="17"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A52" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B52" s="14">
+        <v>320</v>
+      </c>
+      <c r="C52" s="14">
+        <v>10</v>
+      </c>
+      <c r="D52" s="14">
+        <v>275</v>
+      </c>
+      <c r="E52" s="14">
+        <v>400</v>
+      </c>
+      <c r="F52" s="14">
+        <v>250</v>
+      </c>
+      <c r="G52" s="14">
+        <v>5</v>
+      </c>
+      <c r="H52" s="14">
+        <v>19</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>1274</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+        <v>166</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N52" s="17"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A53" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B53" s="14">
+        <v>354</v>
+      </c>
+      <c r="C53" s="14">
+        <v>10</v>
+      </c>
+      <c r="D53" s="14">
+        <v>240</v>
+      </c>
+      <c r="E53" s="14">
+        <v>400</v>
+      </c>
+      <c r="F53" s="14">
+        <v>250</v>
+      </c>
+      <c r="G53" s="14">
+        <v>5</v>
+      </c>
+      <c r="H53" s="14">
+        <v>10</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>1264</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
+        <v>176</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>54</v>
+      </c>
       <c r="N53" s="17"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
@@ -3129,11 +3570,11 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="15" t="str">
-        <f t="shared" ref="I70:I133" si="2">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="J70" s="15" t="str">
-        <f t="shared" ref="J70:J133" si="3">IF(I70="","",1440-I70)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K70" s="16"/>
@@ -3151,11 +3592,11 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I71:I134" si="2">IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
         <v/>
       </c>
       <c r="J71" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J71:J134" si="3">IF(I71="","",1440-I71)</f>
         <v/>
       </c>
       <c r="K71" s="16"/>
@@ -4537,11 +4978,11 @@
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
       <c r="I134" s="15" t="str">
-        <f t="shared" ref="I134:I197" si="4">IF(SUM(B134:F134,H134)=0,"",SUM(B134:F134,H134))</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="J134" s="15" t="str">
-        <f t="shared" ref="J134:J197" si="5">IF(I134="","",1440-I134)</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="K134" s="16"/>
@@ -4559,11 +5000,11 @@
       <c r="G135" s="14"/>
       <c r="H135" s="14"/>
       <c r="I135" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I135:I198" si="4">IF(SUM(B135:F135,H135)=0,"",SUM(B135:F135,H135))</f>
         <v/>
       </c>
       <c r="J135" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="J135:J198" si="5">IF(I135="","",1440-I135)</f>
         <v/>
       </c>
       <c r="K135" s="16"/>
@@ -5945,11 +6386,11 @@
       <c r="G198" s="14"/>
       <c r="H198" s="14"/>
       <c r="I198" s="15" t="str">
-        <f t="shared" ref="I198:I261" si="6">IF(SUM(B198:F198,H198)=0,"",SUM(B198:F198,H198))</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="J198" s="15" t="str">
-        <f t="shared" ref="J198:J261" si="7">IF(I198="","",1440-I198)</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="K198" s="16"/>
@@ -5967,11 +6408,11 @@
       <c r="G199" s="14"/>
       <c r="H199" s="14"/>
       <c r="I199" s="15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="I199:I262" si="6">IF(SUM(B199:F199,H199)=0,"",SUM(B199:F199,H199))</f>
         <v/>
       </c>
       <c r="J199" s="15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="J199:J262" si="7">IF(I199="","",1440-I199)</f>
         <v/>
       </c>
       <c r="K199" s="16"/>
@@ -7353,11 +7794,11 @@
       <c r="G262" s="14"/>
       <c r="H262" s="14"/>
       <c r="I262" s="15" t="str">
-        <f t="shared" ref="I262:I325" si="8">IF(SUM(B262:F262,H262)=0,"",SUM(B262:F262,H262))</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="J262" s="15" t="str">
-        <f t="shared" ref="J262:J325" si="9">IF(I262="","",1440-I262)</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K262" s="16"/>
@@ -7375,11 +7816,11 @@
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
       <c r="I263" s="15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I263:I326" si="8">IF(SUM(B263:F263,H263)=0,"",SUM(B263:F263,H263))</f>
         <v/>
       </c>
       <c r="J263" s="15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="J263:J326" si="9">IF(I263="","",1440-I263)</f>
         <v/>
       </c>
       <c r="K263" s="16"/>
@@ -8761,11 +9202,11 @@
       <c r="G326" s="14"/>
       <c r="H326" s="14"/>
       <c r="I326" s="15" t="str">
-        <f t="shared" ref="I326:I389" si="10">IF(SUM(B326:F326,H326)=0,"",SUM(B326:F326,H326))</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J326" s="15" t="str">
-        <f t="shared" ref="J326:J389" si="11">IF(I326="","",1440-I326)</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="K326" s="16"/>
@@ -8783,11 +9224,11 @@
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
       <c r="I327" s="15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I327:I390" si="10">IF(SUM(B327:F327,H327)=0,"",SUM(B327:F327,H327))</f>
         <v/>
       </c>
       <c r="J327" s="15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="J327:J390" si="11">IF(I327="","",1440-I327)</f>
         <v/>
       </c>
       <c r="K327" s="16"/>
@@ -10169,11 +10610,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="13">IF(I390="","",1440-I390)</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -10191,11 +10632,11 @@
       <c r="G391" s="14"/>
       <c r="H391" s="14"/>
       <c r="I391" s="15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="I391:I401" si="12">IF(SUM(B391:F391,H391)=0,"",SUM(B391:F391,H391))</f>
         <v/>
       </c>
       <c r="J391" s="15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="J391:J401" si="13">IF(I391="","",1440-I391)</f>
         <v/>
       </c>
       <c r="K391" s="16"/>
@@ -10425,12 +10866,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:N4"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <conditionalFormatting sqref="J6:J401">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
@@ -10438,20 +10879,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K401" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K34:K401 K6:K7 K17:K24" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L401" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="K8:K16 L6:L7 L17:L401" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M401" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M401 L8:L16" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated daily logs for dated 18-10-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{26D09376-620A-40D2-825D-D04CFBC51477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94BA0BD0-17FF-45D1-8B2F-21CDB9143657}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{26D09376-620A-40D2-825D-D04CFBC51477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD8C8308-DCA3-447F-B2EA-0AEE8966D1AB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1047,11 +1047,11 @@
         <v>10</v>
       </c>
       <c r="I6" s="12">
-        <f>SUM(B6:F6,H6)</f>
+        <f t="shared" ref="I6:I30" si="0">SUM(B6:F6,H6)</f>
         <v>772</v>
       </c>
       <c r="J6" s="12">
-        <f>1440-I6</f>
+        <f t="shared" ref="J6:J32" si="1">1440-I6</f>
         <v>668</v>
       </c>
       <c r="K6" s="13" t="s">
@@ -1091,11 +1091,11 @@
         <v>15</v>
       </c>
       <c r="I7" s="12">
-        <f>SUM(B7:F7,H7)</f>
+        <f t="shared" si="0"/>
         <v>729</v>
       </c>
       <c r="J7" s="12">
-        <f>1440-I7</f>
+        <f t="shared" si="1"/>
         <v>711</v>
       </c>
       <c r="K7" s="13" t="s">
@@ -1135,11 +1135,11 @@
         <v>25</v>
       </c>
       <c r="I8" s="12">
-        <f>SUM(B8:F8,H8)</f>
+        <f t="shared" si="0"/>
         <v>793</v>
       </c>
       <c r="J8" s="12">
-        <f>1440-I8</f>
+        <f t="shared" si="1"/>
         <v>647</v>
       </c>
       <c r="K8" s="13" t="s">
@@ -1179,11 +1179,11 @@
         <v>8</v>
       </c>
       <c r="I9" s="12">
-        <f>SUM(B9:F9,H9)</f>
+        <f t="shared" si="0"/>
         <v>915</v>
       </c>
       <c r="J9" s="12">
-        <f>1440-I9</f>
+        <f t="shared" si="1"/>
         <v>525</v>
       </c>
       <c r="K9" s="13" t="s">
@@ -1223,11 +1223,11 @@
         <v>11</v>
       </c>
       <c r="I10" s="12">
-        <f>SUM(B10:F10,H10)</f>
+        <f t="shared" si="0"/>
         <v>1326</v>
       </c>
       <c r="J10" s="12">
-        <f>1440-I10</f>
+        <f t="shared" si="1"/>
         <v>114</v>
       </c>
       <c r="K10" s="13" t="s">
@@ -1267,11 +1267,11 @@
         <v>10</v>
       </c>
       <c r="I11" s="12">
-        <f>SUM(B11:F11,H11)</f>
+        <f t="shared" si="0"/>
         <v>1265</v>
       </c>
       <c r="J11" s="12">
-        <f>1440-I11</f>
+        <f t="shared" si="1"/>
         <v>175</v>
       </c>
       <c r="K11" s="13" t="s">
@@ -1311,11 +1311,11 @@
         <v>9</v>
       </c>
       <c r="I12" s="12">
-        <f>SUM(B12:F12,H12)</f>
+        <f t="shared" si="0"/>
         <v>1159</v>
       </c>
       <c r="J12" s="12">
-        <f>1440-I12</f>
+        <f t="shared" si="1"/>
         <v>281</v>
       </c>
       <c r="K12" s="13" t="s">
@@ -1355,11 +1355,11 @@
         <v>15</v>
       </c>
       <c r="I13" s="12">
-        <f>SUM(B13:F13,H13)</f>
+        <f t="shared" si="0"/>
         <v>1261</v>
       </c>
       <c r="J13" s="12">
-        <f>1440-I13</f>
+        <f t="shared" si="1"/>
         <v>179</v>
       </c>
       <c r="K13" s="13" t="s">
@@ -1399,11 +1399,11 @@
         <v>12</v>
       </c>
       <c r="I14" s="12">
-        <f>SUM(B14:F14,H14)</f>
+        <f t="shared" si="0"/>
         <v>1366</v>
       </c>
       <c r="J14" s="12">
-        <f>1440-I14</f>
+        <f t="shared" si="1"/>
         <v>74</v>
       </c>
       <c r="K14" s="13" t="s">
@@ -1443,11 +1443,11 @@
         <v>14</v>
       </c>
       <c r="I15" s="12">
-        <f>SUM(B15:F15,H15)</f>
+        <f t="shared" si="0"/>
         <v>1292</v>
       </c>
       <c r="J15" s="12">
-        <f>1440-I15</f>
+        <f t="shared" si="1"/>
         <v>148</v>
       </c>
       <c r="K15" s="13" t="s">
@@ -1487,11 +1487,11 @@
         <v>10</v>
       </c>
       <c r="I16" s="12">
-        <f>SUM(B16:F16,H16)</f>
+        <f t="shared" si="0"/>
         <v>1080</v>
       </c>
       <c r="J16" s="12">
-        <f>1440-I16</f>
+        <f t="shared" si="1"/>
         <v>360</v>
       </c>
       <c r="K16" s="13" t="s">
@@ -1531,11 +1531,11 @@
         <v>11</v>
       </c>
       <c r="I17" s="12">
-        <f>SUM(B17:F17,H17)</f>
+        <f t="shared" si="0"/>
         <v>1176</v>
       </c>
       <c r="J17" s="12">
-        <f>1440-I17</f>
+        <f t="shared" si="1"/>
         <v>264</v>
       </c>
       <c r="K17" s="13" t="s">
@@ -1575,11 +1575,11 @@
         <v>19</v>
       </c>
       <c r="I18" s="12">
-        <f>SUM(B18:F18,H18)</f>
+        <f t="shared" si="0"/>
         <v>1274</v>
       </c>
       <c r="J18" s="12">
-        <f>1440-I18</f>
+        <f t="shared" si="1"/>
         <v>166</v>
       </c>
       <c r="K18" s="13" t="s">
@@ -1619,11 +1619,11 @@
         <v>10</v>
       </c>
       <c r="I19" s="12">
-        <f>SUM(B19:F19,H19)</f>
+        <f t="shared" si="0"/>
         <v>1264</v>
       </c>
       <c r="J19" s="12">
-        <f>1440-I19</f>
+        <f t="shared" si="1"/>
         <v>176</v>
       </c>
       <c r="K19" s="13" t="s">
@@ -1663,11 +1663,11 @@
         <v>10</v>
       </c>
       <c r="I20" s="12">
-        <f>SUM(B20:F20,H20)</f>
+        <f t="shared" si="0"/>
         <v>1320</v>
       </c>
       <c r="J20" s="12">
-        <f>1440-I20</f>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="K20" s="11" t="s">
@@ -1707,11 +1707,11 @@
         <v>15</v>
       </c>
       <c r="I21" s="12">
-        <f>SUM(B21:F21,H21)</f>
+        <f t="shared" si="0"/>
         <v>1350</v>
       </c>
       <c r="J21" s="12">
-        <f>1440-I21</f>
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
       <c r="K21" s="11" t="s">
@@ -1751,11 +1751,11 @@
         <v>15</v>
       </c>
       <c r="I22" s="12">
-        <f>SUM(B22:F22,H22)</f>
+        <f t="shared" si="0"/>
         <v>1265</v>
       </c>
       <c r="J22" s="12">
-        <f>1440-I22</f>
+        <f t="shared" si="1"/>
         <v>175</v>
       </c>
       <c r="K22" s="11" t="s">
@@ -1795,11 +1795,11 @@
         <v>10</v>
       </c>
       <c r="I23" s="12">
-        <f>SUM(B23:F23,H23)</f>
+        <f t="shared" si="0"/>
         <v>1325</v>
       </c>
       <c r="J23" s="12">
-        <f>1440-I23</f>
+        <f t="shared" si="1"/>
         <v>115</v>
       </c>
       <c r="K23" s="13" t="s">
@@ -1839,11 +1839,11 @@
         <v>10</v>
       </c>
       <c r="I24" s="12">
-        <f>SUM(B24:F24,H24)</f>
+        <f t="shared" si="0"/>
         <v>1070</v>
       </c>
       <c r="J24" s="12">
-        <f>1440-I24</f>
+        <f t="shared" si="1"/>
         <v>370</v>
       </c>
       <c r="K24" s="13" t="s">
@@ -1883,11 +1883,11 @@
         <v>15</v>
       </c>
       <c r="I25" s="12">
-        <f>SUM(B25:F25,H25)</f>
+        <f t="shared" si="0"/>
         <v>930</v>
       </c>
       <c r="J25" s="12">
-        <f>1440-I25</f>
+        <f t="shared" si="1"/>
         <v>510</v>
       </c>
       <c r="K25" s="13" t="s">
@@ -1927,11 +1927,11 @@
         <v>10</v>
       </c>
       <c r="I26" s="12">
-        <f>SUM(B26:F26,H26)</f>
+        <f t="shared" si="0"/>
         <v>950</v>
       </c>
       <c r="J26" s="12">
-        <f>1440-I26</f>
+        <f t="shared" si="1"/>
         <v>490</v>
       </c>
       <c r="K26" s="13" t="s">
@@ -1971,11 +1971,11 @@
         <v>15</v>
       </c>
       <c r="I27" s="12">
-        <f>SUM(B27:F27,H27)</f>
+        <f t="shared" si="0"/>
         <v>1005</v>
       </c>
       <c r="J27" s="12">
-        <f>1440-I27</f>
+        <f t="shared" si="1"/>
         <v>435</v>
       </c>
       <c r="K27" s="13" t="s">
@@ -2015,11 +2015,11 @@
         <v>45</v>
       </c>
       <c r="I28" s="12">
-        <f>SUM(B28:F28,H28)</f>
+        <f t="shared" si="0"/>
         <v>995</v>
       </c>
       <c r="J28" s="12">
-        <f>1440-I28</f>
+        <f t="shared" si="1"/>
         <v>445</v>
       </c>
       <c r="K28" s="13" t="s">
@@ -2059,11 +2059,11 @@
         <v>11</v>
       </c>
       <c r="I29" s="12">
-        <f>SUM(B29:F29,H29)</f>
+        <f t="shared" si="0"/>
         <v>1026</v>
       </c>
       <c r="J29" s="12">
-        <f>1440-I29</f>
+        <f t="shared" si="1"/>
         <v>414</v>
       </c>
       <c r="K29" s="13" t="s">
@@ -2103,11 +2103,11 @@
         <v>11</v>
       </c>
       <c r="I30" s="12">
-        <f>SUM(B30:F30,H30)</f>
+        <f t="shared" si="0"/>
         <v>872</v>
       </c>
       <c r="J30" s="12">
-        <f>1440-I30</f>
+        <f t="shared" si="1"/>
         <v>568</v>
       </c>
       <c r="K30" s="13" t="s">
@@ -2122,35 +2122,91 @@
       <c r="N30" s="14"/>
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
+      <c r="A31" s="10">
+        <v>46312</v>
+      </c>
+      <c r="B31" s="11">
+        <v>430</v>
+      </c>
+      <c r="C31" s="11">
+        <v>20</v>
+      </c>
+      <c r="D31" s="11">
+        <v>160</v>
+      </c>
+      <c r="E31" s="11">
+        <v>400</v>
+      </c>
+      <c r="F31" s="11">
+        <v>240</v>
+      </c>
+      <c r="G31" s="11">
+        <v>4</v>
+      </c>
+      <c r="H31" s="11">
+        <v>15</v>
+      </c>
+      <c r="I31" s="12">
+        <f t="shared" ref="I31:I32" si="2">SUM(B31:F31,H31)</f>
+        <v>1265</v>
+      </c>
+      <c r="J31" s="12">
+        <f t="shared" si="1"/>
+        <v>175</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="L31" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="M31" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="N31" s="14"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="10"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="12"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
-      <c r="M32" s="13"/>
+      <c r="A32" s="10">
+        <v>46313</v>
+      </c>
+      <c r="B32" s="11">
+        <v>440</v>
+      </c>
+      <c r="C32" s="11">
+        <v>25</v>
+      </c>
+      <c r="D32" s="11">
+        <v>100</v>
+      </c>
+      <c r="E32" s="11">
+        <v>350</v>
+      </c>
+      <c r="F32" s="11">
+        <v>0</v>
+      </c>
+      <c r="G32" s="11">
+        <v>0</v>
+      </c>
+      <c r="H32" s="11">
+        <v>15</v>
+      </c>
+      <c r="I32" s="12">
+        <f t="shared" si="2"/>
+        <v>930</v>
+      </c>
+      <c r="J32" s="12">
+        <f t="shared" si="1"/>
+        <v>510</v>
+      </c>
+      <c r="K32" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L32" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="M32" s="13" t="s">
+        <v>56</v>
+      </c>
       <c r="N32" s="14"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
dupdated daily logs dated 22-10-2026
</commit_message>
<xml_diff>
--- a/12620739.xlsx
+++ b/12620739.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc702aa5db0068a/Desktop/daily_logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{26D09376-620A-40D2-825D-D04CFBC51477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD8C8308-DCA3-447F-B2EA-0AEE8966D1AB}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{26D09376-620A-40D2-825D-D04CFBC51477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EF423AC-635A-4105-9A25-006FABCCCCC2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2147,7 +2147,7 @@
         <v>15</v>
       </c>
       <c r="I31" s="12">
-        <f t="shared" ref="I31:I32" si="2">SUM(B31:F31,H31)</f>
+        <f t="shared" ref="I31:I36" si="2">SUM(B31:F31,H31)</f>
         <v>1265</v>
       </c>
       <c r="J31" s="12">
@@ -2210,67 +2210,179 @@
       <c r="N32" s="14"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
+      <c r="A33" s="10">
+        <v>46314</v>
+      </c>
+      <c r="B33" s="11">
+        <v>430</v>
+      </c>
+      <c r="C33" s="11">
+        <v>20</v>
+      </c>
+      <c r="D33" s="11">
+        <v>160</v>
+      </c>
+      <c r="E33" s="11">
+        <v>400</v>
+      </c>
+      <c r="F33" s="11">
+        <v>240</v>
+      </c>
+      <c r="G33" s="11">
+        <v>4</v>
+      </c>
+      <c r="H33" s="11">
+        <v>15</v>
+      </c>
+      <c r="I33" s="12">
+        <f t="shared" si="2"/>
+        <v>1265</v>
+      </c>
+      <c r="J33" s="12">
+        <f t="shared" ref="J33:J36" si="3">1440-I33</f>
+        <v>175</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="L33" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="M33" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="N33" s="14"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="13"/>
-      <c r="L34" s="13"/>
-      <c r="M34" s="13"/>
+      <c r="A34" s="10">
+        <v>46315</v>
+      </c>
+      <c r="B34" s="11">
+        <v>400</v>
+      </c>
+      <c r="C34" s="11">
+        <v>45</v>
+      </c>
+      <c r="D34" s="11">
+        <v>150</v>
+      </c>
+      <c r="E34" s="11">
+        <v>420</v>
+      </c>
+      <c r="F34" s="11">
+        <v>300</v>
+      </c>
+      <c r="G34" s="11">
+        <v>4</v>
+      </c>
+      <c r="H34" s="11">
+        <v>10</v>
+      </c>
+      <c r="I34" s="12">
+        <f t="shared" si="2"/>
+        <v>1325</v>
+      </c>
+      <c r="J34" s="12">
+        <f t="shared" si="3"/>
+        <v>115</v>
+      </c>
+      <c r="K34" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="L34" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M34" s="13" t="s">
+        <v>55</v>
+      </c>
       <c r="N34" s="14"/>
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
+      <c r="A35" s="10">
+        <v>46316</v>
+      </c>
+      <c r="B35" s="11">
+        <v>550</v>
+      </c>
+      <c r="C35" s="11">
+        <v>10</v>
+      </c>
+      <c r="D35" s="11">
+        <v>100</v>
+      </c>
+      <c r="E35" s="11">
+        <v>400</v>
+      </c>
+      <c r="F35" s="11">
+        <v>0</v>
+      </c>
+      <c r="G35" s="11">
+        <v>0</v>
+      </c>
+      <c r="H35" s="11">
+        <v>10</v>
+      </c>
+      <c r="I35" s="12">
+        <f t="shared" si="2"/>
+        <v>1070</v>
+      </c>
+      <c r="J35" s="12">
+        <f t="shared" si="3"/>
+        <v>370</v>
+      </c>
+      <c r="K35" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="L35" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="M35" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="N35" s="14"/>
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="13"/>
-      <c r="M36" s="13"/>
+      <c r="A36" s="10">
+        <v>46317</v>
+      </c>
+      <c r="B36" s="11">
+        <v>440</v>
+      </c>
+      <c r="C36" s="11">
+        <v>25</v>
+      </c>
+      <c r="D36" s="11">
+        <v>100</v>
+      </c>
+      <c r="E36" s="11">
+        <v>350</v>
+      </c>
+      <c r="F36" s="11">
+        <v>0</v>
+      </c>
+      <c r="G36" s="11">
+        <v>0</v>
+      </c>
+      <c r="H36" s="11">
+        <v>15</v>
+      </c>
+      <c r="I36" s="12">
+        <f t="shared" si="2"/>
+        <v>930</v>
+      </c>
+      <c r="J36" s="12">
+        <f t="shared" si="3"/>
+        <v>510</v>
+      </c>
+      <c r="K36" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L36" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="M36" s="13" t="s">
+        <v>56</v>
+      </c>
       <c r="N36" s="14"/>
     </row>
     <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>